<commit_message>
Update carousel log - Topic 4
</commit_message>
<xml_diff>
--- a/carousel-data/carousel-log.xlsx
+++ b/carousel-data/carousel-log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K289"/>
+  <dimension ref="A1:K292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -15004,6 +15004,96 @@
         </is>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Building Trust in Remote Leadership Teams</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>trust-killers</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>remote-trust-2026-04-27</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>7</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>LinkedIn, LinkedIn Page, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Building Trust in Remote Leadership Teams</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>build-trust</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>remote-trust-2026-04-27</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>8</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>LinkedIn, LinkedIn Page, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Building Trust in Remote Leadership Teams</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>remote-rituals</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>remote-trust-2026-04-27</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>8</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>LinkedIn, LinkedIn Page, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>